<commit_message>
update aulas intra 3
</commit_message>
<xml_diff>
--- a/cronograma.xlsx
+++ b/cronograma.xlsx
@@ -3670,7 +3670,10 @@
       <c r="D124" s="5"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D125" s="5"/>
+      <c r="B125" s="3"/>
+      <c r="C125" s="3"/>
+      <c r="D125" s="4"/>
+      <c r="E125" s="3"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="3"/>

</xml_diff>

<commit_message>
biosegurança setembro de 23 para 27
</commit_message>
<xml_diff>
--- a/cronograma.xlsx
+++ b/cronograma.xlsx
@@ -7811,7 +7811,7 @@
         <v>83</v>
       </c>
       <c r="B181" s="9" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C181" s="9" t="s">
         <v>91</v>
@@ -7855,7 +7855,7 @@
         <v>83</v>
       </c>
       <c r="B182" s="9" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C182" s="9" t="s">
         <v>79</v>
@@ -7927,7 +7927,7 @@
         <v>83</v>
       </c>
       <c r="B184" s="9" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C184" s="9" t="s">
         <v>82</v>
@@ -7971,7 +7971,7 @@
         <v>83</v>
       </c>
       <c r="B185" s="9" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C185" s="9" t="s">
         <v>82</v>

</xml_diff>